<commit_message>
Format the excel file
</commit_message>
<xml_diff>
--- a/code/Expiring_Suppliers_Check.xlsx
+++ b/code/Expiring_Suppliers_Check.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Expiring Certifications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Expiring Certifications'!$A$1:$AC$40</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,30 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +58,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,3382 +452,3414 @@
   </sheetPr>
   <dimension ref="A1:AC40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="52" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="43" customWidth="1" min="25" max="25"/>
+    <col width="76" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="38" customWidth="1" min="28" max="28"/>
+    <col width="48" customWidth="1" min="29" max="29"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Approved Supplier</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ID No.</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Select</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Specialty</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Medium +</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>OEM</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dist</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Customer Designated</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ISO9001</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>AS9100D</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>9120 B</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>NADCAP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>17025</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ANSI/NCSL  Z540.3</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>13485</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Phone Number</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Contact</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 24</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 25</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 26</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>List needs to be Finalized and Released</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ACCURATE STEEL TREATING</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>ACCURATE S</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>02/28/25</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>HEAT TREAT</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>HEAT TREATING INCONEL</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>10008 Miller Way South Gate CA 90280</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>562-927-6528</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">david@accuratesteeltreating.com </t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Add Contact Information to each Supplier</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ADEPT FASTENERS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>ADEPT FAST</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>04/28/26</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>HARDWARE</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>FASTENERS</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>27949 Hancock Parkway, Valencia, CA 91355</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>661-257-660</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>Sarah Duenkel</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr">
         <is>
           <t>avanegas@adeptfasteners.com</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ADVANCED METAL FINISHING - SPX SUPPLIER</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>AMF</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>05/31/25</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>ANODIZE, CHEM, CAD</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>ANODIZING, CHEMICAL COATING</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> 2130 March Rd Roseville CA 95747</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>916-910-3117</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>Tom</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">tom@amfservices.net </t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr">
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
         <is>
           <t>Updates to Approved Supplier List:</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>AMERICAN PRECISION ASSEMBLY</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>AMERICAN P</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>03/06/26</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>ASSEMBLY</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>ASSEMBLY</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>5601 Research Dr Huntington Beach CA 92649</t>
         </is>
       </c>
-      <c r="W5" t="n">
+      <c r="W5" s="2" t="n">
         <v>7149038610</v>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="X5" s="2" t="inlineStr">
         <is>
           <t>Steve</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="Y5" s="2" t="inlineStr">
         <is>
           <t>contactus@americanprecisionassembly.com</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr">
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AC5" s="2" t="inlineStr">
         <is>
           <t>Supplier needs to be Determined as Qualified</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ATLAS TESTING</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>ATLAS TEST</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>MATERIAL TESTING</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>MATERIAL TESTING</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr">
         <is>
           <t>9820 6th St Rancho Cucamonga CA 91730</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="W6" s="2" t="inlineStr">
         <is>
           <t>(909) 373-4130</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="X6" s="2" t="inlineStr">
         <is>
           <t>Wendy Valadez</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="Y6" s="2" t="inlineStr">
         <is>
           <t>wendy@atlastesting.com</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>CARR CONSULTING - AS9100</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>CARR CONSU</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>04/23/26</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>AS9100 CONSULTING</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>INTERNAL AUDITS</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>949.306.4354</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t>Lisa/Fred Carr</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="Y7" s="2" t="inlineStr">
         <is>
           <t>fred@carrconsulting.org</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CASTLE METALS</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>CASTLE M</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>09/18/25</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>SST, ALUMINUM</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>14001 Orange Ave Paramount CA 90723</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="W8" s="2" t="inlineStr">
         <is>
           <t>562-259-0209</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="X8" s="2" t="inlineStr">
         <is>
           <t>Chrissy Crerar</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="Y8" s="2" t="inlineStr">
         <is>
           <t>Chrissy crerar@amcastle.com</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>CERTIFIED STEEL TREATING</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>CERT H.T</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>05/31/26</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>HEAT TREAT</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>HEAT TREAT</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t>2454 E 58th St Los Angeles CA 90058</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t>323-583-8711</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="X9" s="2" t="inlineStr">
         <is>
           <t>Darren Kennedy</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Y9" s="2" t="inlineStr">
         <is>
           <t>darren@certifiedsteeltreat.com</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>COAST ALUMINUM</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>COAST ALUM</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>05/11/26</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>10628 Fulton Wells Santa Fe Springs CA 90670</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="W10" s="2" t="inlineStr">
         <is>
           <t>562-946-6061</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="X10" s="2" t="inlineStr">
         <is>
           <t>Joey Blatnik</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="Y10" s="2" t="inlineStr">
         <is>
           <t>joeyb@coastaluminum.com</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>DANCO (Arcadia)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>DANCO ARCA</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>05/31/26</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>ANO, CHEM FILM, PLATING, CHEMICAL PROCESSING</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>TITANIUM ANO</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>44 La Porte St Arcadia CA 91006</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>626-445-3303</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="X11" s="2" t="inlineStr">
         <is>
           <t>George Saunders</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="Y11" s="2" t="inlineStr">
         <is>
           <t>george.s@danco.net</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>DANCO (Santa Ana)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>DANCO</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>05/31/26</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>401 W. Rowland Santa Ana CA 92707</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t>626-445-3303</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t>George Saunders</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t>george.s@danco.net</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">DORAN SPECIALTIES </t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>DORAN SPEC</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>06/27/26</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>HARDWARE</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>FASTENERS</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr">
         <is>
           <t>22855 Savi Ranch Pkwy #D Yorba Linda CA 92887</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="W13" s="2" t="inlineStr">
         <is>
           <t>714-283-3020</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="X13" s="2" t="inlineStr">
         <is>
           <t>Robyn Harrison</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Y13" s="2" t="inlineStr">
         <is>
           <t>robyn@doranspecialties.com</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ELECTROLURGY PLATING </t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>ELECTROLUR</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>05/23/26</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>ELECTROLESS NICKLE</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>ELECTROLESS NICKLE PLATE</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr">
         <is>
           <t>1121 Duryea Ave Irvine CA 92614</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="W14" s="2" t="inlineStr">
         <is>
           <t>949-250-4494</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="X14" s="2" t="inlineStr">
         <is>
           <t>Ty Hilva</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Y14" s="2" t="inlineStr">
         <is>
           <t>sales@electrolurgy.com</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="Z14" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>EMBEE</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>EMBEE</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr">
         <is>
           <t>2136 South Hathaway Street Santa Ana, CA 92705</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="W15" s="2" t="inlineStr">
         <is>
           <t>714-546-9842</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="X15" s="2" t="inlineStr">
         <is>
           <t>Debbie Boone</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Y15" s="2" t="inlineStr">
         <is>
           <t>DebbieB@embee.com</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FASTENERS WEST </t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>FAST WEST</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>12/20/25</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>HARDWARE</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>FASTENERS</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr">
         <is>
           <t>555 W Lambert Rd Ste E Brea CA 92821</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="W16" s="2" t="inlineStr">
         <is>
           <t>714-540-2436</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="X16" s="2" t="inlineStr">
         <is>
           <t>Nelon Surapak</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Y16" s="2" t="inlineStr">
         <is>
           <t>nsurapak@pencomsf.com</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>HADCO METAL TRADING</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>HADCO</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>08/25/26</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">ALUM PLATE / ALUM </t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr">
         <is>
           <t>14088 Borate St Santa Fe Springs CA 90670</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="W17" s="2" t="inlineStr">
         <is>
           <t>310-667-9004</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="X17" s="2" t="inlineStr">
         <is>
           <t>Maly Sun</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Y17" s="2" t="inlineStr">
         <is>
           <t>MalyS@hadco-metal.com</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>HUB METALS &amp; TRADING</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>HUB METALS</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>02/23/26</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>SST, ALUMINUM</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr">
         <is>
           <t>1141 S Acacia Ave, Fullerton, CA 92831</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="W18" s="2" t="inlineStr">
         <is>
           <t>714-871-8020</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="X18" s="2" t="inlineStr">
         <is>
           <t>Casey</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="Y18" s="2" t="inlineStr">
         <is>
           <t>brittneeb@hubmetals.com</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="Z18" s="2" t="inlineStr">
         <is>
           <t>Need to check</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr"/>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>HUDSON TOOL STEEL</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>HUDSON</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>04/03/26</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>HIGH SPEED STEELS</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="2" t="inlineStr">
         <is>
           <t>17871 Park Plaza Dr Ste#135 Cerritos CA 90703</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="W19" s="2" t="inlineStr">
         <is>
           <t>800-966-0411</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="X19" s="2" t="inlineStr">
         <is>
           <t>Bonnie</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Y19" s="2" t="inlineStr">
         <is>
           <t>casales@hudsontoolsteel.com</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr"/>
+      <c r="AA19" s="2" t="inlineStr"/>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">INTEGRAL PRODUCTS INC. </t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>INTEGRAL P</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>05/02/26</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PRIMER </t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>PRIMER FOR INSERT INSTALL</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="2" t="inlineStr">
         <is>
           <t>24045 Frampton Ave Harbor City CA 90710</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="W20" s="2" t="inlineStr">
         <is>
           <t>310-326-8889</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="X20" s="2" t="inlineStr">
         <is>
           <t>Ritchie Suico-Hoyt</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="Y20" s="2" t="inlineStr">
         <is>
           <t>Ritchie@integralproducts.com</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="Z20" s="2" t="inlineStr">
         <is>
           <t>info@integralproducts.com</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
+      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>MARPLES GEARSINC</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>MARPLES</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>02/17/26</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Gears</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>GEARS</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr"/>
+      <c r="V21" s="2" t="inlineStr">
         <is>
           <t>808 W. Santa Anita Street San Gabriel, CA 91776</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="W21" s="2" t="inlineStr">
         <is>
           <t>626.570.1744</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="X21" s="2" t="inlineStr">
         <is>
           <t>Lidia Calderon</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="Y21" s="2" t="inlineStr">
         <is>
           <t>Lidia@marplesgearsinc.com</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr"/>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>METAL SURFACE INC.</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>METAL SURF</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>CHEMICAL PROCESSING</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>CHEMICAL PROCESSING</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr"/>
+      <c r="V22" s="2" t="inlineStr">
         <is>
           <t>6060 Shull Street Bell Gardens CA 90201</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="W22" s="2" t="inlineStr">
         <is>
           <t>562-927-1331</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr">
+      <c r="X22" s="2" t="inlineStr"/>
+      <c r="Y22" s="2" t="inlineStr">
         <is>
           <t>orders@metalsurfaces.com</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr"/>
+      <c r="AA22" s="2" t="inlineStr"/>
+      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>MISTRAS</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>MISTRAS</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr"/>
+      <c r="V23" s="2" t="inlineStr">
         <is>
           <t>8427 Atlantic Ave Cudahy CA 90201</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="W23" s="2" t="inlineStr">
         <is>
           <t>323-583-1653</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="X23" s="2" t="inlineStr">
         <is>
           <t>Shaun Hill</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="Y23" s="2" t="inlineStr">
         <is>
           <t>shaun.hill@mistrasgroup.com</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="Z23" s="2" t="inlineStr">
         <is>
           <t>updated 10/14/24</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr"/>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>MULTICHROME/MICROPLATE</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>MMP</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>05/31/25</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>CHROME, CHEMICAL PROCESSING</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>CHROME</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="2" t="inlineStr">
         <is>
           <t>1013 W. Hillcrest Blvd Inglewood CA 90301</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="W24" s="2" t="inlineStr">
         <is>
           <t>310-417-8381</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="X24" s="2" t="inlineStr">
         <is>
           <t>Tina SanGaspar</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="Y24" s="2" t="inlineStr">
         <is>
           <t>sales@multiplate.com</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr"/>
+      <c r="AB24" s="2" t="inlineStr"/>
+      <c r="AC24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>ND TESTING, INC.</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>ND TEST</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>08/31/26</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>NON-DESTRUCTIVE TESTING</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>NON-DESTRUCTIVE TESTING</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr">
         <is>
           <t>11473 Pacific Avenue, Fontana, CA 92337</t>
         </is>
       </c>
-      <c r="W25" t="inlineStr">
+      <c r="W25" s="2" t="inlineStr">
         <is>
           <t>909.988.4054</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="X25" s="2" t="inlineStr">
         <is>
           <t>QA-Joseph Delgado</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="Y25" s="2" t="inlineStr">
         <is>
           <t>DANT@NDTESTING.COM</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr"/>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>PERFORMANCE TITANIUM GROUP</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>PTG</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>01/27/26</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>TITANIUM MATERIAL</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="2" t="inlineStr">
         <is>
           <t>8025 Silverton Ave San Diego CA 92126</t>
         </is>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="W26" s="2" t="inlineStr">
         <is>
           <t>888-772-8984</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="X26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Sasha Popham </t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
+      <c r="Y26" s="2" t="inlineStr">
         <is>
           <t>spopham@performancetitanium.com</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr"/>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PRECISION ANODIZING AND PLATING </t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>PREC ANOD</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>08/31/26</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>ANODIZE, PASSIVATE, CHEMFILM</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>ANODIZE, CHEM, PASSIVATE</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr">
         <is>
           <t>1601 N. Miller St. Anaheim CA 92806</t>
         </is>
       </c>
-      <c r="W27" t="inlineStr">
+      <c r="W27" s="2" t="inlineStr">
         <is>
           <t>714-996-1601</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="X27" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Anthony </t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
+      <c r="Y27" s="2" t="inlineStr">
         <is>
           <t>anthony@anodizing-plating.com</t>
         </is>
       </c>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr"/>
+      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>PRECISION INSTRUMENT CORRECTIONS</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>PREC INST</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>01/31/26</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">CALIBRATION </t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>INSPECTION TOOL CALIBRATION</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr"/>
+      <c r="V28" s="2" t="inlineStr">
         <is>
           <t>933 Mariner Street Brea CA 92821</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="W28" s="2" t="inlineStr">
         <is>
           <t>714-671-6018</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="X28" s="2" t="inlineStr">
         <is>
           <t>Terrie Klenk</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
+      <c r="Y28" s="2" t="inlineStr">
         <is>
           <t>terrie@picinc.net</t>
         </is>
       </c>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr"/>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>QAP METAL FINISHING</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>QAP</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>NDT</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="2" t="inlineStr">
         <is>
           <t>342 W. 130th Los Angeles CA 90061</t>
         </is>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="W29" s="2" t="inlineStr">
         <is>
           <t>310-327-5201</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="X29" s="2" t="inlineStr">
         <is>
           <t>Bryan Garcia</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="Y29" s="2" t="inlineStr">
         <is>
           <t>david@qapmetalfinishing.com</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AA29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">QUALITY EDM </t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>QUALITYEDM</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>05/31/26</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EDM </t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr"/>
+      <c r="V30" s="2" t="inlineStr">
         <is>
           <t>8025 E. Crystal Dr Anaheim Hills CA 92807</t>
         </is>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="W30" s="2" t="inlineStr">
         <is>
           <t>714-283-9220</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="X30" s="2" t="inlineStr">
         <is>
           <t>Mike Gervais</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
+      <c r="Y30" s="2" t="inlineStr">
         <is>
           <t>qualityedm@aol.com</t>
         </is>
       </c>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr"/>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AA30" s="2" t="inlineStr"/>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>ROLLED ALLOYS</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>ROLLED ALL</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>06/08/26</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">SST / ALUM / TITANIUM </t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr"/>
+      <c r="V31" s="2" t="inlineStr">
         <is>
           <t>4942 W Rosecrans Ave Hawthorne CA 90250</t>
         </is>
       </c>
-      <c r="W31" t="inlineStr">
+      <c r="W31" s="2" t="inlineStr">
         <is>
           <t>800-321-0909</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="X31" s="2" t="inlineStr">
         <is>
           <t>Katrina Ramirez</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
+      <c r="Y31" s="2" t="inlineStr">
         <is>
           <t>kramirez@rolledalloys.com</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="Z31" s="2" t="inlineStr">
         <is>
           <t>Updated 10/15/24 Sales assistance email: region300sales@rolledalloys.com</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr"/>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
+      <c r="AA31" s="2" t="inlineStr"/>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>SEALEZE</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>SEALEZE</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>04/01/26</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>HARDWARE</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>BUSHING</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr"/>
+      <c r="V32" s="2" t="inlineStr">
         <is>
           <t>2350 Salisbury Rd, Richmond, IN 47374</t>
         </is>
       </c>
-      <c r="W32" t="inlineStr">
+      <c r="W32" s="2" t="inlineStr">
         <is>
           <t>800-787-7325</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr">
+      <c r="X32" s="2" t="inlineStr"/>
+      <c r="Y32" s="2" t="inlineStr">
         <is>
           <t>industrial@sealeze.com</t>
         </is>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="Z32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> sealezeorders@sealeze.com</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr"/>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
+      <c r="AA32" s="2" t="inlineStr"/>
+      <c r="AB32" s="2" t="inlineStr"/>
+      <c r="AC32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>SOLAR ATMOSPHERES</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>SOLAR ATMO</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>08/31/26</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>HEAT TREAT</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>HEAT TREATING INCONEL</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="2" t="inlineStr">
         <is>
           <t>8606 Live Oak Ave Fontana CA 92335</t>
         </is>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="W33" s="2" t="inlineStr">
         <is>
           <t>866-559-5994</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="X33" s="2" t="inlineStr">
         <is>
           <t>Frank Trujillo</t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
+      <c r="Y33" s="2" t="inlineStr">
         <is>
           <t>frankt@solaratm.com</t>
         </is>
       </c>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr"/>
+      <c r="AB33" s="2" t="inlineStr"/>
+      <c r="AC33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>SUNSHINE METALS</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>SUNSHINE</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>03/12/25</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr"/>
+      <c r="V34" s="2" t="inlineStr">
         <is>
           <t>1228 Sherborn St Corona CA 92879</t>
         </is>
       </c>
-      <c r="W34" t="inlineStr">
+      <c r="W34" s="2" t="inlineStr">
         <is>
           <t>714-441-8120</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
+      <c r="X34" s="2" t="inlineStr">
         <is>
           <t>Chris Similar</t>
         </is>
       </c>
-      <c r="Y34" t="inlineStr">
+      <c r="Y34" s="2" t="inlineStr">
         <is>
           <t>csimilar@sunshinemetals.com</t>
         </is>
       </c>
-      <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="inlineStr"/>
-      <c r="AB34" t="inlineStr"/>
-      <c r="AC34" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr"/>
+      <c r="AB34" s="2" t="inlineStr"/>
+      <c r="AC34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>THE EDM SHOP</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>EDM</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>08/05/26</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>EDM</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>EDM</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr"/>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr"/>
+      <c r="V35" s="2" t="inlineStr">
         <is>
           <t>1321-B East St Gertrude Place Santa Ana CA 92705</t>
         </is>
       </c>
-      <c r="W35" t="inlineStr">
+      <c r="W35" s="2" t="inlineStr">
         <is>
           <t>714-424-0050</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="X35" s="2" t="inlineStr">
         <is>
           <t>Franz</t>
         </is>
       </c>
-      <c r="Y35" t="inlineStr">
+      <c r="Y35" s="2" t="inlineStr">
         <is>
           <t>franz@theedmshop.com</t>
         </is>
       </c>
-      <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
-      <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="AA35" s="2" t="inlineStr"/>
+      <c r="AB35" s="2" t="inlineStr"/>
+      <c r="AC35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>THERMAL VAC</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>THERMAL VA</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>02/28/26</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Heat Treat</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>TITANIUM H/T</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr"/>
+      <c r="V36" s="2" t="inlineStr">
         <is>
           <t>1221 W. Struck Ave Orange CA 92867</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr">
+      <c r="W36" s="2" t="inlineStr">
         <is>
           <t>714-997-2601</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="X36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Brend Gomez </t>
         </is>
       </c>
-      <c r="Y36" t="inlineStr">
+      <c r="Y36" s="2" t="inlineStr">
         <is>
           <t>jklebau@thermalvac.com</t>
         </is>
       </c>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
-      <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr"/>
+      <c r="AB36" s="2" t="inlineStr"/>
+      <c r="AC36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>THIN METAL SALES, INC.</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>THIN METAL</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>08/08/26</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">THIN MATERIALS </t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr"/>
+      <c r="T37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr"/>
+      <c r="V37" s="2" t="inlineStr">
         <is>
           <t>5721 Schaefer Ave Chino CA 91710</t>
         </is>
       </c>
-      <c r="W37" t="inlineStr">
+      <c r="W37" s="2" t="inlineStr">
         <is>
           <t>909-393-2273</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr">
+      <c r="X37" s="2" t="inlineStr"/>
+      <c r="Y37" s="2" t="inlineStr">
         <is>
           <t>sales@thinmetalsales.com</t>
         </is>
       </c>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
-      <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="AA37" s="2" t="inlineStr"/>
+      <c r="AB37" s="2" t="inlineStr"/>
+      <c r="AC37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>TITANIUM INDUSTRIES</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>TITANIUM</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>04/06/26</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TITANIUM </t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="2" t="inlineStr">
         <is>
           <t>7373 Hunt Ave Garden Grove VA 92841</t>
         </is>
       </c>
-      <c r="W38" t="inlineStr">
+      <c r="W38" s="2" t="inlineStr">
         <is>
           <t>714-895-7756</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
+      <c r="X38" s="2" t="inlineStr">
         <is>
           <t>Patrick Eastman</t>
         </is>
       </c>
-      <c r="Y38" t="inlineStr">
+      <c r="Y38" s="2" t="inlineStr">
         <is>
           <t>peastman@titanium.com</t>
         </is>
       </c>
-      <c r="Z38" t="inlineStr"/>
-      <c r="AA38" t="inlineStr"/>
-      <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="2" t="inlineStr"/>
+      <c r="AC38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>WIRE CUT COMPANY</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>WIRECUT</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>05/08/26</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>WIRE EDM</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>EDM</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr"/>
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="2" t="inlineStr">
         <is>
           <t>6750 Caballero Blvd Buena Park CA 90620</t>
         </is>
       </c>
-      <c r="W39" t="inlineStr">
+      <c r="W39" s="2" t="inlineStr">
         <is>
           <t>714-994-1170</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
+      <c r="X39" s="2" t="inlineStr">
         <is>
           <t>Chris Marks</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
+      <c r="Y39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info@wirecutcompany.com </t>
         </is>
       </c>
-      <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="inlineStr"/>
-      <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr"/>
+      <c r="AB39" s="2" t="inlineStr"/>
+      <c r="AC39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Y&amp;W TECHNOLOGIES</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Y &amp; W</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>02/09/26</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>CHROME PLATE, Ti ANO, PASSIVATE</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>MEDICAL DEVICE FINISHING</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr">
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="2" t="inlineStr">
         <is>
           <t>2883 Directors Cove Memphis TN 38131</t>
         </is>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="W40" s="2" t="inlineStr">
         <is>
           <t>901-396-3380</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr">
+      <c r="X40" s="2" t="inlineStr"/>
+      <c r="Y40" s="2" t="inlineStr">
         <is>
           <t>info@ywtech.com</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="inlineStr"/>
-      <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr"/>
+      <c r="AB40" s="2" t="inlineStr"/>
+      <c r="AC40" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>